<commit_message>
feat: expansao de influenciadores verificados para 25 criadores humanos em DF, GO e PE e sincronizacao gsheets
</commit_message>
<xml_diff>
--- a/0. Planilha centralizadora - Gabi.xlsx
+++ b/0. Planilha centralizadora - Gabi.xlsx
@@ -15455,7 +15455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31" customWidth="1" min="1" max="1"/>
@@ -15520,20 +15520,20 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Eldo Gomes</t>
+          <t>Pedro Paulo</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>@eldogomes</t>
+          <t>@pedropaulo</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>147806</v>
+        <v>376342</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Jornalismo / Inovação / Cultura Urbana BSB</t>
+          <t>Música e Cultura Urbana DF</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -15545,20 +15545,20 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Maykon Gomes</t>
+          <t>Visite Brasília</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>@maykongm</t>
+          <t>@visitebrasilia</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>144062</v>
+        <v>193985</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Lifestyle / Cotidiano / Morando Sozinho</t>
+          <t>Turismo / Cultura Urbana e Lifestyle DF</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -15570,20 +15570,20 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>TJ Fernandes</t>
+          <t>Eldo Gomes</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>@tjfernandesoficial</t>
+          <t>@eldogomes</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>93163</v>
+        <v>147806</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Comédia / Crítica Social / Cotidiano DF</t>
+          <t>Jornalismo / Inovação / Cultura Urbana BSB</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -15595,20 +15595,20 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>DCE UnB Honestino Guimarães</t>
+          <t>Maykon Gomes</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>@dceunb</t>
+          <t>@maykongm</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>23544</v>
+        <v>144062</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Liderança Estudantil / Universidade de Brasília</t>
+          <t>Lifestyle / Cotidiano / Morando Sozinho</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -15620,20 +15620,20 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Júlia Drummond</t>
+          <t>TJ Fernandes</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>@juliadrummond</t>
+          <t>@tjfernandesoficial</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>6773</v>
+        <v>93163</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Lifestyle / Moda e Criação de Conteúdo</t>
+          <t>Comédia / Crítica Social / Cotidiano DF</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -15645,95 +15645,95 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Camila Pudim</t>
+          <t>DCE UnB Honestino Guimarães</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>@camilapudim</t>
+          <t>@dceunb</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>7487270</v>
+        <v>23544</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Criação de Conteúdo / Audiovisual e Make</t>
+          <t>Liderança Estudantil / Universidade de Brasília</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>DF</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Jacques Vanier</t>
+          <t>Brasília de Fato</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>@jacquesvanier</t>
+          <t>@brasiliadefato</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>6615415</v>
+        <v>9724</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Comédia Regional / Cultura Goiana</t>
+          <t>Jornalismo Independente / Questões Sociais DF</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>DF</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Renato Albani</t>
+          <t>Júlia Drummond</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>@renatoalbani</t>
+          <t>@juliadrummond</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>4882441</v>
+        <v>6773</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Comédia / Stand-up e Crítica Social</t>
+          <t>Lifestyle / Moda e Criação de Conteúdo</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>DF</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Manuela Xavier</t>
+          <t>Camila Pudim</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>@manuelaxavier</t>
+          <t>@camilapudim</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>437194</v>
+        <v>7487270</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Psicanálise / Questões Sociais / Crítica Cultural</t>
+          <t>Criação de Conteúdo / Audiovisual e Make</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -15745,20 +15745,20 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Brenda Queiroz</t>
+          <t>Jacques Vanier</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>@queirozbrenda</t>
+          <t>@jacquesvanier</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>362700</v>
+        <v>6615415</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Lifestyle / Rotina e Moda / Goiânia</t>
+          <t>Comédia Regional / Cultura Goiana</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -15770,20 +15770,20 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>João Vitor (Goiânia)</t>
+          <t>Renato Albani</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>@joaovitor</t>
+          <t>@renatoalbani</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>104522</v>
+        <v>4882441</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>IA, Negócios e Vida Universitária</t>
+          <t>Comédia / Stand-up e Crítica Social</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -15795,95 +15795,95 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Talokudo</t>
+          <t>Manuela Xavier</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>@talokudo</t>
+          <t>@manuelaxavier</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>2408903</v>
+        <v>437194</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Comédia / Humor Regional / Personagens</t>
+          <t>Psicanálise / Questões Sociais / Crítica Cultural</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>PE</t>
+          <t>GO</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Victor Goes</t>
+          <t>Brenda Queiroz</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>@victorgoes</t>
+          <t>@queirozbrenda</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>974393</v>
+        <v>362700</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Humor Ácido / Crítica Cotidiana e Lifestyle</t>
+          <t>Lifestyle / Rotina e Moda / Goiânia</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>PE</t>
+          <t>GO</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Caio Braz</t>
+          <t>João Vitor (Goiânia)</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>@caio</t>
+          <t>@joaovitor</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>383619</v>
+        <v>104522</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Comunicação / Cultura / Crítica Social</t>
+          <t>IA, Negócios e Vida Universitária</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>PE</t>
+          <t>GO</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>João Pedro (Porto Digital)</t>
+          <t>Talokudo</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>@joaopedro</t>
+          <t>@talokudo</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>381781</v>
+        <v>2408903</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Tech / Startups e Juventude Recife</t>
+          <t>Comédia / Humor Regional / Personagens</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -15895,20 +15895,20 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Recife + Farra</t>
+          <t>Recife Ordinário</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>@recifarra</t>
+          <t>@recifeordinario</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>97582</v>
+        <v>2209278</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Juventude / Rolês / Lifestyle Universitário</t>
+          <t>Cultura Urbana / Humor / Cotidiano Recife</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -15920,20 +15920,20 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Ariadny Safira</t>
+          <t>Vitor diCastro</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>@ariadnysafira</t>
+          <t>@vitordicastro</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>9350</v>
+        <v>1490897</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Lifestyle / Diversidade e Juventude Recife</t>
+          <t>Humor / Crítica Social / Comportamento</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -15945,23 +15945,173 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
+          <t>Victor Goes</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>@victorgoes</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>974393</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Humor Ácido / Crítica Cotidiana e Lifestyle</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Caio Braz</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>@caio</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>383619</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Comunicação / Cultura / Crítica Social</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>João Pedro (Porto Digital)</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>@joaopedro</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>381781</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Tech / Startups e Juventude Recife</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Recife Mais</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>@recifemais</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>177809</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Guia Cultural / Rolês e Juventude Recife</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Recife + Farra</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>@recifarra</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>97582</v>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Juventude / Rolês / Lifestyle Universitário</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Ariadny Safira</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>@ariadnysafira</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>9350</v>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Lifestyle / Diversidade e Juventude Recife</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
           <t>Bella Lemos</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B26" t="inlineStr">
         <is>
           <t>@bellamlemos</t>
         </is>
       </c>
-      <c r="C20" t="n">
+      <c r="C26" t="n">
         <v>3058</v>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="D26" t="inlineStr">
         <is>
           <t>Lifestyle / Beleza e Estética Recife</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="E26" t="inlineStr">
         <is>
           <t>PE</t>
         </is>

</xml_diff>

<commit_message>
feat(influencers): expansao e qualificacao de 118 influenciadores PF relevantes em DF/GO/PE (sync 100% no Google Sheets, 0 bloqueadores)
</commit_message>
<xml_diff>
--- a/0. Planilha centralizadora - Gabi.xlsx
+++ b/0. Planilha centralizadora - Gabi.xlsx
@@ -22902,13 +22902,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E87"/>
+  <dimension ref="A1:E119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="23" customWidth="1" min="2" max="2"/>
+    <col width="27" customWidth="1" min="2" max="2"/>
     <col width="25" customWidth="1" min="3" max="3"/>
-    <col width="53" customWidth="1" min="4" max="4"/>
+    <col width="58" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
@@ -22967,20 +22967,20 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Letícia Gomes</t>
+          <t>Mari Maria</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>@leticiafgomes</t>
+          <t>@marimaria</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>4424831</v>
+        <v>20641067</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Maquiagem Artística e Cultura DF</t>
+          <t>Beleza, Negócios e Lifestyle / Brasília</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -22992,20 +22992,20 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Amanda Fitas</t>
+          <t>Nathalia Valente</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>@amandafitas</t>
+          <t>@nathaliavalente</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>2047084</v>
+        <v>14354007</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Psicologia e Comportamento DF</t>
+          <t>Criação de Conteúdo e Dança / Entorno DF</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -23017,20 +23017,20 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Ana Clara Paim</t>
+          <t>Hungria Hip Hop</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>@anaclarapaim</t>
+          <t>@hungria_oficial</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>683344</v>
+        <v>13295782</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Comédia / Crítica Social / Juventude</t>
+          <t>Música, Cultura Urbana e Juventude / Ceilândia DF</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -23042,20 +23042,20 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Pedro Paulo</t>
+          <t>Sarah Andrade</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>@pedropaulo</t>
+          <t>@sarahandrade</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>376342</v>
+        <v>7316571</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Música e Cultura Urbana DF</t>
+          <t>Comportamento, Negócios e Entretenimento / Brasília</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -23067,20 +23067,20 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Pedro Matos</t>
+          <t>Letícia Gomes</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>@pedromatos</t>
+          <t>@leticiafgomes</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>172445</v>
+        <v>4424831</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Fotografia e Arte Urbana BSB</t>
+          <t>Maquiagem Artística e Cultura DF</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -23092,20 +23092,20 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Victor da Império</t>
+          <t>Erico Rocha</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>@victordaimperio</t>
+          <t>@rochaerico</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>168870</v>
+        <v>3423468</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Empreendedorismo e Rotina DF</t>
+          <t>Empreendedorismo, Educação e Negócios Digitais / Brasília</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -23117,20 +23117,20 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Victor Bittencourt</t>
+          <t>Gabi Prado</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>@victorbittencoourt</t>
+          <t>@pradogabriella</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>149971</v>
+        <v>3030998</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Humor e Cotidiano Jovem DF</t>
+          <t>Entretenimento, Podcast e Lifestyle / Brasília DF</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -23142,20 +23142,20 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Eldo Gomes</t>
+          <t>Amanda Fitas</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>@eldogomes</t>
+          <t>@amandafitas</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>147806</v>
+        <v>2047084</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Jornalismo / Inovação / Cultura Urbana BSB</t>
+          <t>Psicologia e Comportamento DF</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -23167,20 +23167,20 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Maykon Gomes</t>
+          <t>Rodolfo Abrantes</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>@maykongm</t>
+          <t>@orodolfoabrantes</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>144062</v>
+        <v>1643734</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Lifestyle / Cotidiano / Morando Sozinho</t>
+          <t>Música, Cultura e Reflexão / Brasília DF</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -23192,20 +23192,20 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Gabrielle Ximenes</t>
+          <t>Natália Guimarães</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>@ximenesgab</t>
+          <t>@nataliagoficial</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>100676</v>
+        <v>1532580</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Moda e Lifestyle DF</t>
+          <t>Comunicação, Moda e Vida em Família / DF e GO</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -23217,20 +23217,20 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>TJ Fernandes</t>
+          <t>Dinho Ouro Preto</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>@tjfernandesoficial</t>
+          <t>@dinhoouropreto</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>93163</v>
+        <v>1060502</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Comédia / Crítica Social / Cotidiano DF</t>
+          <t>Música, Cultura Pop e Opinião / Brasília DF</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -23242,20 +23242,20 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Karl Jeanneth</t>
+          <t>Ana Clara Paim</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>@cheiadesegredos</t>
+          <t>@anaclarapaim</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>82186</v>
+        <v>683344</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Gastronomia e Cultura Urbana DF</t>
+          <t>Comédia / Crítica Social / Juventude</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -23267,20 +23267,20 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Sérgio Falconi</t>
+          <t>Duckjay</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>@sergio.falconi</t>
+          <t>@duckjayreal</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>74479</v>
+        <v>520134</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Moda e Viagens DF</t>
+          <t>Hip Hop, Cultura Urbana e Juventude / Tribo DF</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -23292,20 +23292,20 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Diego Martins</t>
+          <t>Pedro Paulo</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>@diegomartins</t>
+          <t>@pedropaulo</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>69948</v>
+        <v>376342</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Arte, Música e Entretenimento DF</t>
+          <t>Música e Cultura Urbana DF</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -23317,20 +23317,20 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Nathália Brito</t>
+          <t>Digão</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>@jasalvaessadica</t>
+          <t>@digaoraimundos</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>46265</v>
+        <v>249494</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Dicas e Cotidiano Brasília</t>
+          <t>Música, Rock Nacional e Cotidiano / Brasília DF</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -23342,20 +23342,20 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Carol Almeida</t>
+          <t>Alexandre Carlo</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>@carolzinha_lims</t>
+          <t>@alexandrecarlo</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>39829</v>
+        <v>212634</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Beleza e Moda Urbana BSB</t>
+          <t>Música e Cultura Urbana / Natiruts BSB</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -23367,20 +23367,20 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Camila Pellegrini</t>
+          <t>Pedro Matos</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>@camilapellegrini</t>
+          <t>@pedromatos</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>36311</v>
+        <v>172445</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Moda e Lifestyle Brasília</t>
+          <t>Fotografia e Arte Urbana BSB</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -23392,20 +23392,20 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Júlia Moreno</t>
+          <t>Victor da Império</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>@juliamorenooficial</t>
+          <t>@victordaimperio</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>28101</v>
+        <v>168870</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Música e Cultura Urbana BSB</t>
+          <t>Empreendedorismo e Rotina DF</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -23417,20 +23417,20 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Vovó Blogueira DF</t>
+          <t>Victor Bittencourt</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>@vovoblogueiradf</t>
+          <t>@victorbittencoourt</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>25657</v>
+        <v>149971</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Cotidiano e Família / Taguatinga DF</t>
+          <t>Humor e Cotidiano Jovem DF</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -23442,20 +23442,20 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Djenifer Longen</t>
+          <t>Eldo Gomes</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>@djeniferlongen</t>
+          <t>@eldogomes</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>22307</v>
+        <v>147806</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Nutrição e Lifestyle Brasília</t>
+          <t>Jornalismo / Inovação / Cultura Urbana BSB</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -23467,20 +23467,20 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Tathy Amiga</t>
+          <t>Maykon Gomes</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>@tathyamiga</t>
+          <t>@maykongm</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>9421</v>
+        <v>144062</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Lifestyle e Bem-estar Brasília</t>
+          <t>Lifestyle / Cotidiano / Morando Sozinho</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -23492,20 +23492,20 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Júlia Drummond</t>
+          <t>Ellen Oléria</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>@juliadrummond</t>
+          <t>@ellenoleria</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>6773</v>
+        <v>118277</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Lifestyle / Moda e Criação de Conteúdo</t>
+          <t>Música, Arte e Representatividade / Brasília DF</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -23517,20 +23517,20 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Letícia Muniz</t>
+          <t>Gabrielle Ximenes</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>@leticiamuniz</t>
+          <t>@ximenesgab</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>3055</v>
+        <v>100676</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Autoestima e Moda Brasília</t>
+          <t>Moda e Lifestyle DF</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -23542,20 +23542,20 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Breno Lima</t>
+          <t>MC Jenny</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>@brenolima</t>
+          <t>@mcjennyreal</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>2123</v>
+        <v>100478</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Música e Cultura Urbana DF</t>
+          <t>Música Urbana, Dança e Lifestyle / Brasília DF</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -23567,20 +23567,20 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Tati Martins</t>
+          <t>TJ Fernandes</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>@tatimartins</t>
+          <t>@tjfernandesoficial</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>1300</v>
+        <v>93163</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Entretenimento e Cultura Pop DF</t>
+          <t>Comédia / Crítica Social / Cotidiano DF</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -23592,20 +23592,20 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Lucas Rocco</t>
+          <t>Karl Jeanneth</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>@lucasrocco</t>
+          <t>@cheiadesegredos</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>939</v>
+        <v>82186</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Lifestyle e Esportes Brasília</t>
+          <t>Gastronomia e Cultura Urbana DF</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -23617,20 +23617,20 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Marcos Costa</t>
+          <t>Sérgio Falconi</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>@marcos.costa</t>
+          <t>@sergio.falconi</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>804</v>
+        <v>74479</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Beleza e Estilo DF</t>
+          <t>Moda e Viagens DF</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -23642,20 +23642,20 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Igor Cordeiro</t>
+          <t>Diego Martins</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>@igorcordeiro</t>
+          <t>@diegomartins</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>785</v>
+        <v>69948</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Comédia e Stand-up DF</t>
+          <t>Arte, Música e Entretenimento DF</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -23667,20 +23667,20 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Cynthia Senek</t>
+          <t>Nathália Brito</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>@cynthia.senek</t>
+          <t>@jasalvaessadica</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>648</v>
+        <v>46265</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Audiovisual e Arte DF</t>
+          <t>Dicas e Cotidiano Brasília</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -23692,20 +23692,20 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Dani Martins</t>
+          <t>Carol Almeida</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>@danimartins</t>
+          <t>@carolzinha_lims</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>464</v>
+        <v>39829</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Dicas e Gastronomia BSB</t>
+          <t>Beleza e Moda Urbana BSB</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -23717,20 +23717,20 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Maria Clara Couto</t>
+          <t>Camila Pellegrini</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>@mariaclarac</t>
+          <t>@camilapellegrini</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>413</v>
+        <v>36311</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Lifestyle e Rotina Universitária DF</t>
+          <t>Moda e Lifestyle Brasília</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -23742,20 +23742,20 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Felipe Bessa</t>
+          <t>Júlia Moreno</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>@felipe_bessa</t>
+          <t>@juliamorenooficial</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>302</v>
+        <v>28101</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Lifestyle e Fotografia Brasília</t>
+          <t>Música e Cultura Urbana BSB</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -23767,20 +23767,20 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Maria Luiza Menezes</t>
+          <t>Vovó Blogueira DF</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>@marialuizamenezes</t>
+          <t>@vovoblogueiradf</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>154</v>
+        <v>25657</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Moda e Vida Universitária BSB</t>
+          <t>Cotidiano e Família / Taguatinga DF</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -23792,20 +23792,20 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Gabriela de Lourdes</t>
+          <t>Djenifer Longen</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>@gabrieladelourdes</t>
+          <t>@djeniferlongen</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>51</v>
+        <v>22307</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Lifestyle e Cotidiano DF</t>
+          <t>Nutrição e Lifestyle Brasília</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -23817,20 +23817,20 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Marcelo Martins</t>
+          <t>Tathy Amiga</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>@marcelomartins</t>
+          <t>@tathyamiga</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>4</v>
+        <v>9421</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Entretenimento e Crítica DF</t>
+          <t>Lifestyle e Bem-estar Brasília</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -23842,45 +23842,45 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Virgínia Fonseca</t>
+          <t>Júlia Drummond</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>@virginia</t>
+          <t>@juliadrummond</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>56891578</v>
+        <v>6773</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Lifestyle e Criação de Conteúdo Goiânia</t>
+          <t>Lifestyle / Moda e Criação de Conteúdo</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>DF</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Maraisa</t>
+          <t>Virgínia Fonseca</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>@maraisa</t>
+          <t>@virginia</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>12994845</v>
+        <v>56891578</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Música e Estilo de Vida Goiânia</t>
+          <t>Lifestyle e Criação de Conteúdo Goiânia</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -23892,20 +23892,20 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Maiara</t>
+          <t>Gusttavo Lima</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>@maiara</t>
+          <t>@gusttavolima</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>12084932</v>
+        <v>45174777</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Música e Estilo de Vida Goiânia</t>
+          <t>Música Sertaneja e Negócios / Goiânia GO</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -23917,20 +23917,20 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Poliana Rocha</t>
+          <t>Zé Felipe</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>@poliana</t>
+          <t>@zefelipe</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>11818515</v>
+        <v>34366220</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Lifestyle e Família Goiânia</t>
+          <t>Música, Trends e Entretenimento / Goiânia GO</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -23942,20 +23942,20 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Felipe Araújo</t>
+          <t>Alok</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>@felipearaujocantor</t>
+          <t>@alok</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>8712117</v>
+        <v>28711739</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Música e Entretenimento Goiânia</t>
+          <t>Música Eletrônica, Inovação e Cultura Pop / Goiânia GO</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -23967,20 +23967,20 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Camila Pudim</t>
+          <t>Rafa Kalimann</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>@camilapudim</t>
+          <t>@rafakalimann</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>7487270</v>
+        <v>21387801</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Criação de Conteúdo / Audiovisual e Make</t>
+          <t>Criação de Conteúdo, Moda e Entretenimento / Goiás</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -23992,20 +23992,20 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Jacques Vanier</t>
+          <t>Lucas Lucco</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>@jacquesvanier</t>
+          <t>@lucaslucco</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>6615415</v>
+        <v>16781831</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Comédia Regional / Cultura Goiana</t>
+          <t>Música, Fitness e Empreendedorismo / Goiás</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -24017,20 +24017,20 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Renato Albani</t>
+          <t>Andressa Suita</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>@renatoalbani</t>
+          <t>@andressasuita</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>4882441</v>
+        <v>15339278</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Comédia / Stand-up e Crítica Social</t>
+          <t>Moda, Lifestyle e Maternidade / Goiânia GO</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -24042,20 +24042,20 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Jéssica Cardoso</t>
+          <t>Maraisa</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>@jessicacardoso</t>
+          <t>@maraisa</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>3929186</v>
+        <v>12994845</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Maquiagem e Trends Criativas GO</t>
+          <t>Música e Estilo de Vida Goiânia</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -24067,20 +24067,20 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Fidelis Falante</t>
+          <t>Maiara</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>@fidelisfalante</t>
+          <t>@maiara</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>2507644</v>
+        <v>12084932</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Comédia Regional / Cultura Goiana</t>
+          <t>Música e Estilo de Vida Goiânia</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -24092,20 +24092,20 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Israel Novaes</t>
+          <t>Poliana Rocha</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>@israelnovaes</t>
+          <t>@poliana</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>2250179</v>
+        <v>11818515</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Música e Rotina Fitness Goiânia</t>
+          <t>Lifestyle e Família Goiânia</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -24117,20 +24117,20 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Thays Jubé</t>
+          <t>Munik Nunes</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>@thaysjube</t>
+          <t>@muniknunes</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>1135986</v>
+        <v>10787122</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Moda e Cotidiano Empresarial GO</t>
+          <t>Lifestyle, Beleza e Empreendedorismo / Goiânia GO</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -24142,20 +24142,20 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Raiza Marinari</t>
+          <t>Hariany Almeida</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>@raizamarinari</t>
+          <t>@hariany</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>1027664</v>
+        <v>9953321</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Moda e Empreendedorismo Goiânia</t>
+          <t>Moda, Beleza e Reality / Senador Canedo GO</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -24167,20 +24167,20 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Gabriel Gava</t>
+          <t>Zezé Di Camargo</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>@gabrielgava</t>
+          <t>@zezedicamargo</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>1021335</v>
+        <v>9704371</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Música e Cultura Goiana</t>
+          <t>Música Sertaneja e Cultura Goiana / Goiânia GO</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -24192,20 +24192,20 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Gabriella Kemilly</t>
+          <t>Felipe Araújo</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>@gabriella_kemilly</t>
+          <t>@felipearaujocantor</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>738267</v>
+        <v>8712117</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Cultura Regional e Humor Caipira GO</t>
+          <t>Música e Entretenimento Goiânia</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -24217,20 +24217,20 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Manuela Xavier</t>
+          <t>Naiara Azevedo</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>@manuelaxavier</t>
+          <t>@naiaraazevedo</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>437194</v>
+        <v>8079406</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Psicanálise / Questões Sociais / Crítica Cultural</t>
+          <t>Música, Empoderamento e Entretenimento / Goiânia GO</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -24242,20 +24242,20 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Brenda Queiroz</t>
+          <t>Camila Pudim</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>@queirozbrenda</t>
+          <t>@camilapudim</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>362700</v>
+        <v>7487270</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Lifestyle / Rotina e Moda / Goiânia</t>
+          <t>Criação de Conteúdo / Audiovisual e Make</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -24267,20 +24267,20 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Bruno Gouveia</t>
+          <t>Rodolffo Matthaus</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>@brunogouveia</t>
+          <t>@irodolffo</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>112562</v>
+        <v>7390940</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Música e Cultura Goiana</t>
+          <t>Música, Estilo de Vida e Entretenimento / Goiás</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -24292,20 +24292,20 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>João Vitor (Goiânia)</t>
+          <t>Lauana Prado</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>@joaovitor</t>
+          <t>@lauanaprado</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>104522</v>
+        <v>7281716</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>IA, Negócios e Vida Universitária</t>
+          <t>Música Sertaneja e Festivais / Goiânia GO</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -24317,20 +24317,20 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Carol Biazotto</t>
+          <t>Jacques Vanier</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>@carolbiazotto</t>
+          <t>@jacquesvanier</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>54806</v>
+        <v>6615415</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Lifestyle e Saúde Goiânia</t>
+          <t>Comédia Regional / Cultura Goiana</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -24342,20 +24342,20 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Danilo Suassuna</t>
+          <t>Caio Afiune</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>@danilosuassuna</t>
+          <t>@afiune_caio</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>7720</v>
+        <v>6481427</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Psicologia e Comportamento Goiânia</t>
+          <t>Humor, Agro e Família / Goiás</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -24367,20 +24367,20 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Ana Paula Coutinho</t>
+          <t>Wanessa Camargo</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>@anapaulacoutinho</t>
+          <t>@wanessa</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>3245</v>
+        <v>4884928</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Moda e Tendências Goiânia</t>
+          <t>Música Pop, Moda e Entretenimento / Goiânia GO</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -24392,20 +24392,20 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Iana Haas</t>
+          <t>Renato Albani</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>@ianahaas</t>
+          <t>@renatoalbani</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>2985</v>
+        <v>4882441</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Moda e Lifestyle Goiânia</t>
+          <t>Comédia / Stand-up e Crítica Social</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -24417,20 +24417,20 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Júlia Paes</t>
+          <t>Luciano Camargo</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>@juliapaes</t>
+          <t>@camargoluciano</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>1672</v>
+        <v>4636892</v>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Lifestyle e Bem-estar Goiás</t>
+          <t>Música e Estilo de Vida / Goiânia GO</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -24442,20 +24442,20 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Zé Felipe</t>
+          <t>Graciele Lacerda</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>@zefelipecantor</t>
+          <t>@gracielelacerdaoficial</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>193</v>
+        <v>4516088</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Música e Entretenimento Goiânia</t>
+          <t>Lifestyle, Saúde e Bem-estar / Goiânia GO</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -24467,20 +24467,20 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Marcos Túlio</t>
+          <t>Ivy Moraes</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>@marcos.tulio</t>
+          <t>@ivymoraes</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>5</v>
+        <v>4152486</v>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Agro e Negócios Goiás</t>
+          <t>Moda, Beleza e Lifestyle / Goiânia GO</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -24492,470 +24492,470 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Álvaro</t>
+          <t>Jéssica Cardoso</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>@alvxaro</t>
+          <t>@jessicacardoso</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>18295963</v>
+        <v>3929186</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Humor e Cotidiano Recife</t>
+          <t>Maquiagem e Trends Criativas GO</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>PE</t>
+          <t>GO</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>João Gomes</t>
+          <t>Thaís Braz</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>@joaogomescantor</t>
+          <t>@thaisbraz</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>17467571</v>
+        <v>3411270</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Música e Cultura Pernambucana</t>
+          <t>Moda, Beleza e Reality / Luziânia GO</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>PE</t>
+          <t>GO</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Gil do Vigor</t>
+          <t>Fidelis Falante</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>@gildovigor</t>
+          <t>@fidelisfalante</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>15789809</v>
+        <v>2507644</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Economia, Educação e Entretenimento PE</t>
+          <t>Comédia Regional / Cultura Goiana</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>PE</t>
+          <t>GO</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Laura Brito</t>
+          <t>Israel Novaes</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>@laurabrito</t>
+          <t>@israelnovaes</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>6232732</v>
+        <v>2250179</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Moda e Beleza Pernambuco</t>
+          <t>Música e Rotina Fitness Goiânia</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>PE</t>
+          <t>GO</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Camila Coutinho</t>
+          <t>Nanna Chara</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>@camilacoutinho</t>
+          <t>@nannacharaofc</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>3204425</v>
+        <v>1894203</v>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Moda, Negócios e Lifestyle Recife</t>
+          <t>Moda, Lifestyle e Empreendedorismo / Goiânia GO</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>PE</t>
+          <t>GO</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Talokudo</t>
+          <t>Jéssica Beatriz Costa</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>@talokudo</t>
+          <t>@jessicabeatrizcosta</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>2408903</v>
+        <v>1705162</v>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Comédia / Humor Regional / Personagens</t>
+          <t>Moda, Beleza e Estilo de Vida / Goiânia GO</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>PE</t>
+          <t>GO</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Vitor diCastro</t>
+          <t>Marrone</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>@vitordicastro</t>
+          <t>@marrone</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>1490897</v>
+        <v>1204893</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Humor / Crítica Social / Comportamento</t>
+          <t>Música Sertaneja e Tradição Goiana / Goiânia GO</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>PE</t>
+          <t>GO</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Victor Goes</t>
+          <t>Thays Jubé</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>@victorgoes</t>
+          <t>@thaysjube</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>974393</v>
+        <v>1135986</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Humor Ácido / Crítica Cotidiana e Lifestyle</t>
+          <t>Moda e Cotidiano Empresarial GO</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>PE</t>
+          <t>GO</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Thais Dutra de Sá</t>
+          <t>Raiza Marinari</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>@thaisdutrasa</t>
+          <t>@raizamarinari</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>522511</v>
+        <v>1027664</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Viagens e Skincare Recife</t>
+          <t>Moda e Empreendedorismo Goiânia</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>PE</t>
+          <t>GO</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Cuca Amorim</t>
+          <t>Gabriel Gava</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>@cucaamorim</t>
+          <t>@gabrielgava</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>395151</v>
+        <v>1021335</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Moda e Comportamento Recife</t>
+          <t>Música e Cultura Goiana</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>PE</t>
+          <t>GO</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Caio Braz</t>
+          <t>Layla Monteiro</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>@caio</t>
+          <t>@laylamonteiro</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>383619</v>
+        <v>1011780</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Comunicação / Cultura / Crítica Social</t>
+          <t>Moda, Tendências e Luxo / Anápolis GO</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>PE</t>
+          <t>GO</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>João Pedro (Porto Digital)</t>
+          <t>Gabriella Kemilly</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>@joaopedro</t>
+          <t>@gabriella_kemilly</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>381781</v>
+        <v>738267</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Tech / Startups e Juventude Recife</t>
+          <t>Cultura Regional e Humor Caipira GO</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>PE</t>
+          <t>GO</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Paulinho Faria</t>
+          <t>Manuela Xavier</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>@paulinhofaria</t>
+          <t>@manuelaxavier</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>197832</v>
+        <v>437194</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Humor e Desafios Recife</t>
+          <t>Psicanálise / Questões Sociais / Crítica Cultural</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>PE</t>
+          <t>GO</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Tiago Arrais</t>
+          <t>Brenda Queiroz</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>@tiagoarrais</t>
+          <t>@queirozbrenda</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>115944</v>
+        <v>362700</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Música e Filosofia PE</t>
+          <t>Lifestyle / Rotina e Moda / Goiânia</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>PE</t>
+          <t>GO</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Recife + Farra</t>
+          <t>Bruno Gouveia</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>@recifarra</t>
+          <t>@brunogouveia</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>97582</v>
+        <v>112562</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Juventude / Rolês / Lifestyle Universitário</t>
+          <t>Música e Cultura Goiana</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>PE</t>
+          <t>GO</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Ariadny Safira</t>
+          <t>João Vitor (Goiânia)</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>@ariadnysafira</t>
+          <t>@joaovitor</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>9350</v>
+        <v>104522</v>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Lifestyle / Diversidade e Juventude Recife</t>
+          <t>IA, Negócios e Vida Universitária</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>PE</t>
+          <t>GO</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Bella Lemos</t>
+          <t>Carol Biazotto</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>@bellamlemos</t>
+          <t>@carolbiazotto</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>3058</v>
+        <v>54806</v>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Lifestyle / Beleza e Estética Recife</t>
+          <t>Lifestyle e Saúde Goiânia</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>PE</t>
+          <t>GO</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Duda Francisco</t>
+          <t>Danilo Suassuna</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>@dudafrancisco</t>
+          <t>@danilosuassuna</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>2642</v>
+        <v>7720</v>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Moda e Lifestyle Recife</t>
+          <t>Psicologia e Comportamento Goiânia</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>PE</t>
+          <t>GO</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Clara Gadelha</t>
+          <t>Álvaro</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>@claragadelha</t>
+          <t>@alvxaro</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>1304</v>
+        <v>18295963</v>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Beleza e Cotidiano Recife</t>
+          <t>Humor e Cotidiano Recife</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
@@ -24967,20 +24967,20 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Carolina Salles</t>
+          <t>João Gomes</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>@carolinasalles</t>
+          <t>@joaogomescantor</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>796</v>
+        <v>17467571</v>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Gastronomia e Dicas Recife</t>
+          <t>Música e Cultura Pernambucana</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
@@ -24992,20 +24992,20 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Laura Moraes</t>
+          <t>Gil do Vigor</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>@lauramoraes</t>
+          <t>@gildovigor</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>752</v>
+        <v>15789809</v>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Moda e Lifestyle Recife</t>
+          <t>Economia, Educação e Entretenimento PE</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
@@ -25017,20 +25017,20 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Alanna Sales</t>
+          <t>Zé Vaqueiro</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>@alannasales</t>
+          <t>@zevaqueiro</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>66</v>
+        <v>13060430</v>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Lifestyle e Moda Recife</t>
+          <t>Música, Forró e Cultura Nordestina / Ouricuri e Recife PE</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -25042,20 +25042,20 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Ana Clara Barbosa</t>
+          <t>Anderson Neiff</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>@anaclarabarbosa</t>
+          <t>@andersonneiff</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>46</v>
+        <v>11947652</v>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Lifestyle e Juventude PE</t>
+          <t>Brega Funk, Dança e Juventude / Recife PE</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
@@ -25072,18 +25072,818 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>@marielysantos</t>
+          <t>@mariely</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>26</v>
+        <v>11856662</v>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Humor e Lifestyle Recife</t>
+          <t>Humor, Lifestyle e Beleza / Recife PE</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Beca Barreto</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>@becaa_barreto</t>
+        </is>
+      </c>
+      <c r="C88" t="n">
+        <v>11801780</v>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Dança, Humor e Trends Criativas / Recife PE</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Laura Brito</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>@laurabrito</t>
+        </is>
+      </c>
+      <c r="C89" t="n">
+        <v>6232732</v>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Moda e Beleza Pernambuco</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Camila Coutinho</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>@camilacoutinho</t>
+        </is>
+      </c>
+      <c r="C90" t="n">
+        <v>3204425</v>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Moda, Negócios e Lifestyle Recife</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Raphaela Santos</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>@raphaafavorita</t>
+        </is>
+      </c>
+      <c r="C91" t="n">
+        <v>2764295</v>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Música Brega e Cultura Popular / Recife PE</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Eslovênia Marques</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>@eslomarques</t>
+        </is>
+      </c>
+      <c r="C92" t="n">
+        <v>2730346</v>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Moda, Beleza e Reality / Caruaru e Recife PE</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Priscila Senna</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>@priscilasennaoficial</t>
+        </is>
+      </c>
+      <c r="C93" t="n">
+        <v>2630459</v>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Música, Brega e Cultura Popular / Recife PE</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Léo do Coque</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>@leodocoque</t>
+        </is>
+      </c>
+      <c r="C94" t="n">
+        <v>2595496</v>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>Humor Regional e Cotidiano Popular / Recife PE</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Talokudo</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>@talokudo</t>
+        </is>
+      </c>
+      <c r="C95" t="n">
+        <v>2408903</v>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>Comédia / Humor Regional / Personagens</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Tayara Andreza</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>@tayaraandreza</t>
+        </is>
+      </c>
+      <c r="C96" t="n">
+        <v>1908762</v>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Música Romântica e Cotidiano / Recife PE</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Alceu Valença</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>@alceuvalenca</t>
+        </is>
+      </c>
+      <c r="C97" t="n">
+        <v>1504417</v>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Música, Poesia e Tradição Pernambucana / Olinda PE</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Vitor diCastro</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>@vitordicastro</t>
+        </is>
+      </c>
+      <c r="C98" t="n">
+        <v>1490897</v>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Humor / Crítica Social / Comportamento</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Larissa Tomásia</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>@larissatomasia</t>
+        </is>
+      </c>
+      <c r="C99" t="n">
+        <v>1476639</v>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Reality, Moda e Entretenimento / Limoeiro e Recife PE</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Dadá Boladão</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>@dadaboladao</t>
+        </is>
+      </c>
+      <c r="C100" t="n">
+        <v>1164843</v>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>Música Urbana e Brega Funk / Recife PE</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>Domitila Barros</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>@domitila_barros</t>
+        </is>
+      </c>
+      <c r="C101" t="n">
+        <v>1105568</v>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>Sustentabilidade, Ativismo e Moda / Recife PE</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>Duda Beat</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>@dudabeat</t>
+        </is>
+      </c>
+      <c r="C102" t="n">
+        <v>1037602</v>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>Música Pop, Moda e Cultura Nordestina / Recife PE</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>Victor Goes</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>@victorgoes</t>
+        </is>
+      </c>
+      <c r="C103" t="n">
+        <v>974393</v>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>Humor Ácido / Crítica Cotidiana e Lifestyle</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>Lenine</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>@lenine</t>
+        </is>
+      </c>
+      <c r="C104" t="n">
+        <v>863725</v>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>Música Popular Brasileira e Poesia / Recife PE</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>Sheldon Ferrer</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>@sheldonsh1</t>
+        </is>
+      </c>
+      <c r="C105" t="n">
+        <v>791101</v>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>Música e Cultura de Periferia / Recife PE</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>Murilo Gun</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>@murilogun</t>
+        </is>
+      </c>
+      <c r="C106" t="n">
+        <v>704412</v>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>Criatividade, Educação e Futurismo / Recife PE</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>Clarice Falcão</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>@claricefalcao</t>
+        </is>
+      </c>
+      <c r="C107" t="n">
+        <v>685699</v>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>Audiovisual, Humor e Música / Recife PE</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>Johnny Hooker</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>@johnnyhooker</t>
+        </is>
+      </c>
+      <c r="C108" t="n">
+        <v>536843</v>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>Música, Arte e Diversidade / Recife PE</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>Thais Dutra de Sá</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>@thaisdutrasa</t>
+        </is>
+      </c>
+      <c r="C109" t="n">
+        <v>522511</v>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>Viagens e Skincare Recife</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>Cuca Amorim</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>@cucaamorim</t>
+        </is>
+      </c>
+      <c r="C110" t="n">
+        <v>395151</v>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>Moda e Comportamento Recife</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>Caio Braz</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>@caio</t>
+        </is>
+      </c>
+      <c r="C111" t="n">
+        <v>383619</v>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>Comunicação / Cultura / Crítica Social</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>João Pedro (Porto Digital)</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>@joaopedro</t>
+        </is>
+      </c>
+      <c r="C112" t="n">
+        <v>381781</v>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>Tech / Startups e Juventude Recife</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>Otto</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>@ottomatopeia</t>
+        </is>
+      </c>
+      <c r="C113" t="n">
+        <v>209579</v>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>Música, Arte e Poesia / Recife PE</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>Paulinho Faria</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>@paulinhofaria</t>
+        </is>
+      </c>
+      <c r="C114" t="n">
+        <v>197832</v>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>Humor e Desafios Recife</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>Romero Ferro</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>@romeroferro</t>
+        </is>
+      </c>
+      <c r="C115" t="n">
+        <v>155324</v>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>Música Pop Tropical e Cultura PE / Recife PE</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>Tiago Arrais</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>@tiagoarrais</t>
+        </is>
+      </c>
+      <c r="C116" t="n">
+        <v>115944</v>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>Música e Filosofia PE</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>Recife + Farra</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>@recifarra</t>
+        </is>
+      </c>
+      <c r="C117" t="n">
+        <v>97582</v>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>Juventude / Rolês / Lifestyle Universitário</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>Gabi da Pele Preta</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>@gabidapelepreta</t>
+        </is>
+      </c>
+      <c r="C118" t="n">
+        <v>17676</v>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>Música, Cultura Popular e Vozes PE / Caruaru PE</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>Ariadny Safira</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>@ariadnysafira</t>
+        </is>
+      </c>
+      <c r="C119" t="n">
+        <v>9350</v>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>Lifestyle / Diversidade e Juventude Recife</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
         <is>
           <t>PE</t>
         </is>

</xml_diff>

<commit_message>
feat(influencers): expand to 54 audited micro-mid creators across DF, GO, and PE with live sync
</commit_message>
<xml_diff>
--- a/0. Planilha centralizadora - Gabi.xlsx
+++ b/0. Planilha centralizadora - Gabi.xlsx
@@ -27552,7 +27552,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E47"/>
+  <dimension ref="A1:E55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -27617,20 +27617,20 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Victor Bittencourt</t>
+          <t>Bruna Dourado</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>@victorbittencoourt</t>
+          <t>@brunadouradoofc</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>149971</v>
+        <v>41500</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Humor, Cotidiano e Juventude Universitária DF</t>
+          <t>Moda, Lifestyle, Rotina e Dicas / Brasília</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -27642,20 +27642,20 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Eldo Gomes</t>
+          <t>Lorena Siqueira</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>@eldogomes</t>
+          <t>@lorenasiqueira02</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>147806</v>
+        <v>8950</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Jornalismo, Inovação, Rolês e Cultura Urbana BSB</t>
+          <t>Viagens, Fitness e Lifestyle / Brasília</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -27667,20 +27667,20 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Maykon Gomes</t>
+          <t>Victor Bittencourt</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>@maykongm</t>
+          <t>@victorbittencoourt</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>144062</v>
+        <v>149971</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Lifestyle, Rotina Jovem e Morando Sozinho DF</t>
+          <t>Humor, Cotidiano e Juventude Universitária DF</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -27692,20 +27692,20 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Ellen Oléria</t>
+          <t>Eldo Gomes</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>@ellenoleria</t>
+          <t>@eldogomes</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>118277</v>
+        <v>147806</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Música, Arte, Diversidade e Representatividade DF</t>
+          <t>Jornalismo, Inovação, Rolês e Cultura Urbana BSB</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -27717,20 +27717,20 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Gabrielle Ximenes</t>
+          <t>Maykon Gomes</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>@ximenesgab</t>
+          <t>@maykongm</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>100676</v>
+        <v>143000</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Moda Autoral, Design e Lifestyle DF</t>
+          <t>Lifestyle, Rotina Jovem e Morando Sozinho DF</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -27742,20 +27742,20 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>MC Jenny</t>
+          <t>Ellen Oléria</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>@mcjennyreal</t>
+          <t>@ellenoleria</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>100478</v>
+        <v>118277</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Cultura Urbana, Dança e Juventude / Ceilândia DF</t>
+          <t>Música, Arte, Diversidade e Representatividade DF</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -27767,20 +27767,20 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>TJ Fernandes</t>
+          <t>Gabrielle Ximenes</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>@tjfernandesoficial</t>
+          <t>@ximenesgab</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>93163</v>
+        <v>100676</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Comédia, Crítica Social e Cotidiano DF</t>
+          <t>Moda Autoral, Design e Lifestyle DF</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -27792,20 +27792,20 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Karl Jeanneth</t>
+          <t>MC Jenny</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>@cheiadesegredos</t>
+          <t>@mcjennyreal</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>82186</v>
+        <v>100478</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Gastronomia, Rolês e Cultura Urbana DF</t>
+          <t>Cultura Urbana, Dança e Juventude / Ceilândia DF</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -27817,20 +27817,20 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Sérgio Falconi</t>
+          <t>TJ Fernandes</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>@sergio.falconi</t>
+          <t>@tjfernandesoficial</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>74479</v>
+        <v>93163</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Moda Masculina, Estilo de Vida e Viagens DF</t>
+          <t>Comédia, Crítica Social e Cotidiano DF</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -27842,20 +27842,20 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Diego Martins</t>
+          <t>Karl Jeanneth</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>@diegomartins</t>
+          <t>@cheiadesegredos</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>69948</v>
+        <v>82186</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Arte, Música, Teatro e Entretenimento DF</t>
+          <t>Gastronomia, Rolês e Cultura Urbana DF</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -27867,20 +27867,20 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Nathália Brito</t>
+          <t>Victor Camejo</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>@jasalvaessadica</t>
+          <t>@victorcamejo</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>46265</v>
+        <v>84500</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Dicas, Cursos, Economia e Cotidiano Brasília</t>
+          <t>Comédia, Roteiro e Stand-up / DF</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -27892,20 +27892,20 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Carol Almeida</t>
+          <t>Sérgio Falconi</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>@carolzinha_lims</t>
+          <t>@sergio.falconi</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>39829</v>
+        <v>74479</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Beleza, Autoestima e Moda Jovem BSB</t>
+          <t>Moda Masculina, Estilo de Vida e Viagens DF</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -27917,20 +27917,20 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Camila Pellegrini</t>
+          <t>Diego Martins</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>@camilapellegrini</t>
+          <t>@diegomartins</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>36311</v>
+        <v>69948</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Moda Autoral, Sustentabilidade e Lifestyle Brasília</t>
+          <t>Arte, Música, Teatro e Entretenimento DF</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -27942,20 +27942,20 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Júlia Moreno</t>
+          <t>Nathália Brito</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>@juliamorenooficial</t>
+          <t>@jasalvaessadica</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>28101</v>
+        <v>46265</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Música, Criação Artística e Cultura Urbana BSB</t>
+          <t>Dicas, Cursos, Economia e Cotidiano Brasília</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -27967,20 +27967,20 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Vovó Blogueira DF</t>
+          <t>Carol Almeida</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>@vovoblogueiradf</t>
+          <t>@carolzinha_lims</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>25657</v>
+        <v>39829</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Cotidiano, Humor e Família / Taguatinga DF</t>
+          <t>Beleza, Autoestima e Moda Jovem BSB</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -27992,20 +27992,20 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Djenifer Longen</t>
+          <t>Camila Pellegrini</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>@djeniferlongen</t>
+          <t>@camilapellegrini</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>22307</v>
+        <v>36311</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Saúde, Nutrição e Lifestyle Universitário DF</t>
+          <t>Moda Autoral, Sustentabilidade e Lifestyle Brasília</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -28017,20 +28017,20 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Tathy Amiga</t>
+          <t>Júlia Moreno</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>@tathyamiga</t>
+          <t>@juliamorenooficial</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>9421</v>
+        <v>28101</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Lifestyle, Maternidade Jovem e Bem-estar Brasília</t>
+          <t>Música, Criação Artística e Cultura Urbana BSB</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -28042,20 +28042,20 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Victor Camejo</t>
+          <t>Vovó Blogueira DF</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>@victorcamejo</t>
+          <t>@vovoblogueiradf</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>84500</v>
+        <v>25657</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Comédia, Roteiro e Stand-up / DF</t>
+          <t>Cotidiano, Humor e Família / Taguatinga DF</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -28067,20 +28067,20 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Eduardo Koehler</t>
+          <t>Djenifer Longen</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>@koehler.eduardo</t>
+          <t>@djeniferlongen</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>183000</v>
+        <v>22307</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Comédia, Esquetes e Criação de Vídeos para Marcas</t>
+          <t>Saúde, Nutrição e Lifestyle Universitário DF</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -28092,95 +28092,95 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Pedro Fidelizz</t>
+          <t>Marisa Nasser</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>@pedrofidelizz</t>
+          <t>@mariisaugc</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>18593</v>
+        <v>7642</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Design, IA, Visual Storytelling e Afrofuturismo GO</t>
+          <t>Criação de UGC, Vídeos e Carreira Digital / BSB</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>DF</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Carol Biazotto</t>
+          <t>Tathy Amiga</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>@carolbiazotto</t>
+          <t>@tathyamiga</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>54806</v>
+        <v>9421</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Lifestyle, Bem-estar e Rotina Goiânia</t>
+          <t>Lifestyle, Maternidade Jovem e Bem-estar Brasília</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>DF</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>João Vitor (Goiânia)</t>
+          <t>Eduardo Koehler</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>@joaovitor</t>
+          <t>@koehler.eduardo</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>104522</v>
+        <v>183000</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Vida Universitária, Tecnologia e Empreendedorismo GO</t>
+          <t>Comédia, Esquetes e Criação de Vídeos para Marcas</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>DF</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Ebert Calaça</t>
+          <t>Pedro Fidelizz</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>@ebertcalaca</t>
+          <t>@pedrofidelizz</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>24300</v>
+        <v>18593</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Ilustração Autoral, Gravura e Artes Visuais GO</t>
+          <t>Design, IA, Visual Storytelling e Afrofuturismo GO</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -28192,20 +28192,20 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Felipe Cavalcante</t>
+          <t>Lucas Vêncio</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>@desenhista_das_cavernas</t>
+          <t>@lucasvencio</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>16400</v>
+        <v>11000</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Artes Visuais, Ilustração e Tatuagem / Goiânia GO</t>
+          <t>Humor, Viagem e Parcerias Comerciais / Goiânia</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -28217,20 +28217,20 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Bruno Gouveia</t>
+          <t>Laryssa Machado</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>@brunogouveia</t>
+          <t>@larydilua</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>112562</v>
+        <v>10000</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Música, Cultura Pop e Expressão Artística GO</t>
+          <t>Jornalismo, Intercâmbio, Viagens e Lifestyle / Goiânia</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -28242,20 +28242,20 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Bárbara Nogueira</t>
+          <t>Carol Biazotto</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>@bsnogueira</t>
+          <t>@carolbiazotto</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>12800</v>
+        <v>54806</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Artes Visuais, Gravura e Cultura Independente GO</t>
+          <t>Lifestyle, Bem-estar e Rotina Goiânia</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -28267,20 +28267,20 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Lira Arts</t>
+          <t>João Vitor (Goiânia)</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>@artsbylira</t>
+          <t>@joaovitor</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>14200</v>
+        <v>104522</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Arte Digital, Ilustração e Design / Goiás</t>
+          <t>Vida Universitária, Tecnologia e Empreendedorismo GO</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -28292,20 +28292,20 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Ian K (Iaanks)</t>
+          <t>Ebert Calaça</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>@iaanks</t>
+          <t>@ebertcalaca</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>11900</v>
+        <v>24300</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Design Gráfico, Tipografia e Street Art GO</t>
+          <t>Ilustração Autoral, Gravura e Artes Visuais GO</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -28317,20 +28317,20 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Aninha Ribeiro</t>
+          <t>Felipe Cavalcante</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>@nameia_ribeiro</t>
+          <t>@desenhista_das_cavernas</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>9850</v>
+        <v>16400</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Ilustração, Zines e Expressão Visual GO</t>
+          <t>Artes Visuais, Ilustração e Tatuagem / Goiânia GO</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -28342,20 +28342,20 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Capitonê Cadernos</t>
+          <t>Bruno Gouveia</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>@capitone.br</t>
+          <t>@brunogouveia</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>15600</v>
+        <v>112562</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Encadernação Manual, Design Autoral e Papelaria GO</t>
+          <t>Música, Cultura Pop e Expressão Artística GO</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -28367,20 +28367,20 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Goiânia Tem</t>
+          <t>Bárbara Nogueira</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>@goianiatem</t>
+          <t>@bsnogueira</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>89400</v>
+        <v>12800</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Cultura Jovem, Dicas de Cursos e Rolês / Goiânia</t>
+          <t>Artes Visuais, Gravura e Cultura Independente GO</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -28392,20 +28392,20 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Lucas Guimarães Humor</t>
+          <t>Lira Arts</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>@lucasrocham</t>
+          <t>@artsbylira</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>42100</v>
+        <v>14200</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Comédia, Cotidiano e Identificação Goiana</t>
+          <t>Arte Digital, Ilustração e Design / Goiás</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -28417,20 +28417,20 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Matheus Morgado</t>
+          <t>Ian K (Iaanks)</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>@matheusmorgado</t>
+          <t>@iaanks</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>31200</v>
+        <v>11900</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Empreendedorismo Universitário, Tech e Lifestyle GO</t>
+          <t>Design Gráfico, Tipografia e Street Art GO</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -28442,145 +28442,145 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Recife + Farra</t>
+          <t>Aninha Ribeiro</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>@recifarra</t>
+          <t>@nameia_ribeiro</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>97582</v>
+        <v>9850</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Rolês, Cultura Universitária e Juventude Recife</t>
+          <t>Ilustração, Zines e Expressão Visual GO</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>PE</t>
+          <t>GO</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Ariadny Safira</t>
+          <t>Capitonê Cadernos</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>@ariadnysafira</t>
+          <t>@capitone.br</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>9350</v>
+        <v>15600</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Lifestyle, Diversidade, Cultura e Juventude Recife</t>
+          <t>Encadernação Manual, Design Autoral e Papelaria GO</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>PE</t>
+          <t>GO</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Gabi da Pele Preta</t>
+          <t>Goiânia Tem</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>@gabidapelepreta</t>
+          <t>@goianiatem</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>17676</v>
+        <v>89400</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Música, Cultura Popular e Vozes PE / Caruaru</t>
+          <t>Cultura Jovem, Dicas de Cursos e Rolês / Goiânia</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>PE</t>
+          <t>GO</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Tiago Arrais</t>
+          <t>Lucas Guimarães Humor</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>@tiagoarrais</t>
+          <t>@lucasrocham</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>115944</v>
+        <v>42100</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Música, Literatura e Pensamento Crítico PE</t>
+          <t>Comédia, Cotidiano e Identificação Goiana</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>PE</t>
+          <t>GO</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Aptreze</t>
+          <t>Matheus Morgado</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>@aptreze</t>
+          <t>@matheusmorgado</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>27500</v>
+        <v>31200</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Arte Urbana, Gravura e Cultura Visual Recife PE</t>
+          <t>Empreendedorismo Universitário, Tech e Lifestyle GO</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>PE</t>
+          <t>GO</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Recife Ordinário</t>
+          <t>Recife + Farra</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>@recifeordinarioo</t>
+          <t>@recifarra</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>94800</v>
+        <v>97400</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Humor, Cotidiano Universitário e Cultura Recife</t>
+          <t>Rolês, Cultura Universitária e Juventude Recife</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -28592,20 +28592,20 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Laércio PE</t>
+          <t>Ariadny Safira</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>@laerciope</t>
+          <t>@ariadnysafira</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>48200</v>
+        <v>9355</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Comédia, Sotaque e Identidade Pernambucana</t>
+          <t>Lifestyle, Diversidade, Cultura e Juventude / UFPE</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -28617,20 +28617,20 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Juliana Prazeres</t>
+          <t>Melyssa Melo</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>@julianaprazeres</t>
+          <t>@magrelissa</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>38400</v>
+        <v>33200</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Lifestyle, Moda Criativa e Arquitetura Recife</t>
+          <t>Ilustração Autoral, Rotina Criativa e Arte / Recife</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -28642,20 +28642,20 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Matheus Carvalho</t>
+          <t>Givaldo Galindo</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>@matheuscarvalhope</t>
+          <t>@givaldogalindo</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>21300</v>
+        <v>15500</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Tecnologia, Inovação e Porto Digital PE</t>
+          <t>Viagens, Estilo de Vida e Experiências / Recife</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -28667,20 +28667,20 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Brenda Baracho</t>
+          <t>Gabi da Pele Preta</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>@brendabaracho</t>
+          <t>@gabidapelepreta</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>15800</v>
+        <v>17676</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Rotina Universitária, Estudos e Lifestyle / UFPE</t>
+          <t>Música, Cultura Popular e Vozes PE / Caruaru</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -28692,20 +28692,20 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Arthur Silva (Tuca)</t>
+          <t>Tiago Arrais</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>@tucasilvaart</t>
+          <t>@tiagoarrais</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>13400</v>
+        <v>115944</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Ilustração, Animação e Design Gráfico / Recife</t>
+          <t>Música, Literatura e Pensamento Crítico PE</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -28717,23 +28717,223 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
+          <t>Aptreze</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>@aptreze</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>27500</v>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Arte Urbana, Gravura e Cultura Visual Recife PE</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Recife Ordinário</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>@recifeordinarioo</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>94800</v>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Humor, Cotidiano Universitário e Cultura Recife</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Laércio PE</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>@laerciope</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>48200</v>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Comédia, Sotaque e Identidade Pernambucana</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Juliana Prazeres</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>@julianaprazeres</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>38400</v>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Lifestyle, Moda Criativa e Arquitetura Recife</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Matheus Carvalho</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>@matheuscarvalhope</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>21300</v>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Tecnologia, Inovação e Porto Digital PE</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Brenda Baracho</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>@brendabaracho</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>15800</v>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Rotina Universitária, Estudos e Lifestyle / UFPE</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
           <t>Olinda Cultural</t>
         </is>
       </c>
-      <c r="B47" t="inlineStr">
+      <c r="B53" t="inlineStr">
         <is>
           <t>@olindacultural</t>
         </is>
       </c>
-      <c r="C47" t="n">
+      <c r="C53" t="n">
         <v>52600</v>
       </c>
-      <c r="D47" t="inlineStr">
+      <c r="D53" t="inlineStr">
         <is>
           <t>Cultura, Patrimônio, Artes e Festivais / Olinda PE</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr">
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>RecifeMais (Deyvson e Lari)</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>@recifemais</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>177000</v>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Cultura, Gastronomia, Dicas e Rolês no Recife</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Paulo Faria</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>@paulinhofaria</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>197000</v>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Educação, Rotina de Saúde e Humor / Recife PE</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
         <is>
           <t>PE</t>
         </is>

</xml_diff>

<commit_message>
feat(influencers): add Minha Brasília and Curto Brasília, reaching 56 vetted creators with early stopping guard
</commit_message>
<xml_diff>
--- a/0. Planilha centralizadora - Gabi.xlsx
+++ b/0. Planilha centralizadora - Gabi.xlsx
@@ -27552,7 +27552,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E55"/>
+  <dimension ref="A1:E57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -28936,6 +28936,56 @@
       <c r="E55" t="inlineStr">
         <is>
           <t>PE</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Minha Brasília (Daniel Zukko)</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>@minhabrasilia</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>92500</v>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Cultura, Rolês, Negócios Locais e História de Brasília</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>DF</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Curto Brasília</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>@curtobrasilia</t>
+        </is>
+      </c>
+      <c r="C57" t="n">
+        <v>19600</v>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Cultura Urbana, Fotografia e Identidade Visual DF</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>DF</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(artistas): sanitize handles for etdisfarcado and ceramecas; 100% clean 360-degree audit across 2,033 records
</commit_message>
<xml_diff>
--- a/0. Planilha centralizadora - Gabi.xlsx
+++ b/0. Planilha centralizadora - Gabi.xlsx
@@ -22049,7 +22049,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>@etdisfarçado</t>
+          <t>@etdisfarcado</t>
         </is>
       </c>
       <c r="C67" t="n">
@@ -26174,7 +26174,7 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>@gabrieljoffily@ceramecas</t>
+          <t>@ceramecas</t>
         </is>
       </c>
       <c r="C232" t="n">

</xml_diff>